<commit_message>
fix(ga): sinkronisasi dinamis keterangan subtext card Penerima Transaksi Terbesar (Ivan terhubung ke Material Proyek Atap Futsal, bukan teks statis UKS SD), dan lengkapi vendor riil Oktober
</commit_message>
<xml_diff>
--- a/static/JURNAL_PENGAJUAN_26.27_LENGKAP_TERVALIDASI.xlsx
+++ b/static/JURNAL_PENGAJUAN_26.27_LENGKAP_TERVALIDASI.xlsx
@@ -9255,7 +9255,11 @@
         <v>120000000</v>
       </c>
       <c r="G153" s="11" t="n"/>
-      <c r="H153" s="11" t="n"/>
+      <c r="H153" s="11" t="inlineStr">
+        <is>
+          <t>Devzar</t>
+        </is>
+      </c>
       <c r="I153" s="19">
         <f>F153</f>
         <v/>
@@ -9304,7 +9308,11 @@
         <v>4500000</v>
       </c>
       <c r="G154" s="11" t="n"/>
-      <c r="H154" s="11" t="n"/>
+      <c r="H154" s="11" t="inlineStr">
+        <is>
+          <t>Masdik</t>
+        </is>
+      </c>
       <c r="I154" s="15" t="n"/>
       <c r="J154" s="15" t="n"/>
       <c r="K154" s="15" t="n"/>
@@ -9350,7 +9358,11 @@
         <v>2000000</v>
       </c>
       <c r="G155" s="11" t="n"/>
-      <c r="H155" s="11" t="n"/>
+      <c r="H155" s="11" t="inlineStr">
+        <is>
+          <t>Masdik</t>
+        </is>
+      </c>
       <c r="I155" s="15" t="n"/>
       <c r="J155" s="15" t="n"/>
       <c r="K155" s="15" t="n"/>
@@ -9396,7 +9408,11 @@
         <v>3322500</v>
       </c>
       <c r="G156" s="11" t="n"/>
-      <c r="H156" s="11" t="n"/>
+      <c r="H156" s="11" t="inlineStr">
+        <is>
+          <t>Rinni</t>
+        </is>
+      </c>
       <c r="I156" s="19">
         <f>F156</f>
         <v/>
@@ -9445,7 +9461,11 @@
         <v>367500</v>
       </c>
       <c r="G157" s="11" t="n"/>
-      <c r="H157" s="11" t="n"/>
+      <c r="H157" s="11" t="inlineStr">
+        <is>
+          <t>Rinni</t>
+        </is>
+      </c>
       <c r="I157" s="19">
         <f>F157</f>
         <v/>
@@ -9494,7 +9514,11 @@
         <v>2000000</v>
       </c>
       <c r="G158" s="11" t="n"/>
-      <c r="H158" s="11" t="n"/>
+      <c r="H158" s="11" t="inlineStr">
+        <is>
+          <t>Rinni</t>
+        </is>
+      </c>
       <c r="I158" s="15" t="n"/>
       <c r="J158" s="15" t="n"/>
       <c r="K158" s="15" t="n"/>
@@ -9540,7 +9564,11 @@
         <v>730000</v>
       </c>
       <c r="G159" s="11" t="n"/>
-      <c r="H159" s="11" t="n"/>
+      <c r="H159" s="11" t="inlineStr">
+        <is>
+          <t>Eko</t>
+        </is>
+      </c>
       <c r="I159" s="19">
         <f>F159</f>
         <v/>
@@ -9589,7 +9617,11 @@
         <v>1560000</v>
       </c>
       <c r="G160" s="11" t="n"/>
-      <c r="H160" s="11" t="n"/>
+      <c r="H160" s="11" t="inlineStr">
+        <is>
+          <t>Eko</t>
+        </is>
+      </c>
       <c r="I160" s="19">
         <f>F160</f>
         <v/>
@@ -9638,7 +9670,11 @@
         <v>1490000</v>
       </c>
       <c r="G161" s="11" t="n"/>
-      <c r="H161" s="11" t="n"/>
+      <c r="H161" s="11" t="inlineStr">
+        <is>
+          <t>Eko</t>
+        </is>
+      </c>
       <c r="I161" s="19">
         <f>F161</f>
         <v/>
@@ -9736,7 +9772,11 @@
         <v>57925000</v>
       </c>
       <c r="G163" s="11" t="n"/>
-      <c r="H163" s="11" t="n"/>
+      <c r="H163" s="11" t="inlineStr">
+        <is>
+          <t>Susi</t>
+        </is>
+      </c>
       <c r="I163" s="19">
         <f>F163</f>
         <v/>
@@ -9785,7 +9825,11 @@
         <v>1958294</v>
       </c>
       <c r="G164" s="11" t="n"/>
-      <c r="H164" s="11" t="n"/>
+      <c r="H164" s="11" t="inlineStr">
+        <is>
+          <t>Susi</t>
+        </is>
+      </c>
       <c r="I164" s="19">
         <f>F164</f>
         <v/>
@@ -9883,7 +9927,11 @@
         <v>3220000</v>
       </c>
       <c r="G166" s="11" t="n"/>
-      <c r="H166" s="11" t="n"/>
+      <c r="H166" s="11" t="inlineStr">
+        <is>
+          <t>Cahaya Alam</t>
+        </is>
+      </c>
       <c r="I166" s="19">
         <f>F166</f>
         <v/>
@@ -9981,7 +10029,11 @@
         <v>16628392</v>
       </c>
       <c r="G168" s="11" t="n"/>
-      <c r="H168" s="11" t="n"/>
+      <c r="H168" s="11" t="inlineStr">
+        <is>
+          <t>Rinni</t>
+        </is>
+      </c>
       <c r="I168" s="19">
         <f>F168</f>
         <v/>
@@ -10030,7 +10082,11 @@
         <v>15661549</v>
       </c>
       <c r="G169" s="11" t="n"/>
-      <c r="H169" s="11" t="n"/>
+      <c r="H169" s="11" t="inlineStr">
+        <is>
+          <t>Rinni</t>
+        </is>
+      </c>
       <c r="I169" s="19">
         <f>F169</f>
         <v/>
@@ -10079,7 +10135,11 @@
         <v>1018875</v>
       </c>
       <c r="G170" s="11" t="n"/>
-      <c r="H170" s="11" t="n"/>
+      <c r="H170" s="11" t="inlineStr">
+        <is>
+          <t>Rinni</t>
+        </is>
+      </c>
       <c r="I170" s="19">
         <f>F170</f>
         <v/>
@@ -10226,7 +10286,11 @@
         <v>5185000</v>
       </c>
       <c r="G173" s="11" t="n"/>
-      <c r="H173" s="11" t="n"/>
+      <c r="H173" s="11" t="inlineStr">
+        <is>
+          <t>Rinni</t>
+        </is>
+      </c>
       <c r="I173" s="19">
         <f>F173</f>
         <v/>
@@ -10275,7 +10339,11 @@
         <v>1045000</v>
       </c>
       <c r="G174" s="11" t="n"/>
-      <c r="H174" s="11" t="n"/>
+      <c r="H174" s="11" t="inlineStr">
+        <is>
+          <t>Bengkel Mobil</t>
+        </is>
+      </c>
       <c r="I174" s="19">
         <f>F174</f>
         <v/>
@@ -10373,7 +10441,11 @@
         <v>12765000</v>
       </c>
       <c r="G176" s="11" t="n"/>
-      <c r="H176" s="11" t="n"/>
+      <c r="H176" s="11" t="inlineStr">
+        <is>
+          <t>Maxindo</t>
+        </is>
+      </c>
       <c r="I176" s="19">
         <f>F176</f>
         <v/>
@@ -10422,7 +10494,11 @@
         <v>10000000</v>
       </c>
       <c r="G177" s="11" t="n"/>
-      <c r="H177" s="11" t="n"/>
+      <c r="H177" s="11" t="inlineStr">
+        <is>
+          <t>Devyzar Syam</t>
+        </is>
+      </c>
       <c r="I177" s="19">
         <f>F177</f>
         <v/>
@@ -10471,7 +10547,11 @@
         <v>1080000</v>
       </c>
       <c r="G178" s="11" t="n"/>
-      <c r="H178" s="11" t="n"/>
+      <c r="H178" s="11" t="inlineStr">
+        <is>
+          <t>Eko</t>
+        </is>
+      </c>
       <c r="I178" s="19">
         <f>F178</f>
         <v/>
@@ -10520,7 +10600,11 @@
         <v>1589400</v>
       </c>
       <c r="G179" s="11" t="n"/>
-      <c r="H179" s="11" t="n"/>
+      <c r="H179" s="11" t="inlineStr">
+        <is>
+          <t>Hannochs</t>
+        </is>
+      </c>
       <c r="I179" s="19">
         <f>F179</f>
         <v/>
@@ -10569,7 +10653,11 @@
         <v>1206000</v>
       </c>
       <c r="G180" s="11" t="n"/>
-      <c r="H180" s="11" t="n"/>
+      <c r="H180" s="11" t="inlineStr">
+        <is>
+          <t>Cahaya Alam</t>
+        </is>
+      </c>
       <c r="I180" s="19">
         <f>F180</f>
         <v/>
@@ -10667,7 +10755,11 @@
         <v>4546000</v>
       </c>
       <c r="G182" s="11" t="n"/>
-      <c r="H182" s="11" t="n"/>
+      <c r="H182" s="11" t="inlineStr">
+        <is>
+          <t>Masdik</t>
+        </is>
+      </c>
       <c r="I182" s="19">
         <f>F182</f>
         <v/>
@@ -10716,7 +10808,11 @@
         <v>2295000</v>
       </c>
       <c r="G183" s="11" t="n"/>
-      <c r="H183" s="11" t="n"/>
+      <c r="H183" s="11" t="inlineStr">
+        <is>
+          <t>Ariyati</t>
+        </is>
+      </c>
       <c r="I183" s="19">
         <f>F183</f>
         <v/>

</xml_diff>

<commit_message>
fix(ga): lengkapi nilai terhitung pada kolom digunakan dan sinkronisasi Row 40 Termin Futsal Misbahudin Rp 20M
</commit_message>
<xml_diff>
--- a/static/JURNAL_PENGAJUAN_26.27_LENGKAP_TERVALIDASI.xlsx
+++ b/static/JURNAL_PENGAJUAN_26.27_LENGKAP_TERVALIDASI.xlsx
@@ -637,13 +637,11 @@
           <t>Mail</t>
         </is>
       </c>
-      <c r="I3" s="19">
-        <f>F3</f>
-        <v/>
-      </c>
-      <c r="J3" s="19">
-        <f>F3-I3</f>
-        <v/>
+      <c r="I3" s="19" t="n">
+        <v>4920000</v>
+      </c>
+      <c r="J3" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K3" s="15" t="n"/>
       <c r="L3" s="15" t="n"/>
@@ -697,13 +695,11 @@
           <t>Mail</t>
         </is>
       </c>
-      <c r="I4" s="19">
-        <f>F4</f>
-        <v/>
-      </c>
-      <c r="J4" s="19">
-        <f>F4-I4</f>
-        <v/>
+      <c r="I4" s="19" t="n">
+        <v>18400000</v>
+      </c>
+      <c r="J4" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K4" s="15" t="n"/>
       <c r="L4" s="15" t="n"/>
@@ -757,13 +753,11 @@
           <t xml:space="preserve">Eko </t>
         </is>
       </c>
-      <c r="I5" s="19">
-        <f>F5</f>
-        <v/>
-      </c>
-      <c r="J5" s="19">
-        <f>F5-I5</f>
-        <v/>
+      <c r="I5" s="19" t="n">
+        <v>1502500</v>
+      </c>
+      <c r="J5" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K5" s="15" t="n"/>
       <c r="L5" s="15" t="n"/>
@@ -820,9 +814,8 @@
       <c r="I6" s="16" t="n">
         <v>3988400</v>
       </c>
-      <c r="J6" s="19">
-        <f>F6-I6</f>
-        <v/>
+      <c r="J6" s="19" t="n">
+        <v>511600</v>
       </c>
       <c r="K6" s="15" t="n"/>
       <c r="L6" s="15" t="n"/>
@@ -879,9 +872,8 @@
       <c r="I7" s="16" t="n">
         <v>2266380</v>
       </c>
-      <c r="J7" s="19">
-        <f>F7-I7</f>
-        <v/>
+      <c r="J7" s="19" t="n">
+        <v>233620</v>
       </c>
       <c r="K7" s="15" t="n"/>
       <c r="L7" s="15" t="n"/>
@@ -935,13 +927,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I8" s="19">
-        <f>F8</f>
-        <v/>
-      </c>
-      <c r="J8" s="19">
-        <f>F8-I8</f>
-        <v/>
+      <c r="I8" s="19" t="n">
+        <v>3322500</v>
+      </c>
+      <c r="J8" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K8" s="15" t="n"/>
       <c r="L8" s="15" t="n"/>
@@ -995,13 +985,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I9" s="19">
-        <f>F9</f>
-        <v/>
-      </c>
-      <c r="J9" s="19">
-        <f>F9-I9</f>
-        <v/>
+      <c r="I9" s="19" t="n">
+        <v>367500</v>
+      </c>
+      <c r="J9" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K9" s="15" t="n"/>
       <c r="L9" s="15" t="n"/>
@@ -1058,9 +1046,8 @@
       <c r="I10" s="16" t="n">
         <v>1183500</v>
       </c>
-      <c r="J10" s="19">
-        <f>F10-I10</f>
-        <v/>
+      <c r="J10" s="19" t="n">
+        <v>816500</v>
       </c>
       <c r="K10" s="15" t="n"/>
       <c r="L10" s="15" t="n"/>
@@ -1114,13 +1101,11 @@
           <t xml:space="preserve">Eko </t>
         </is>
       </c>
-      <c r="I11" s="19">
-        <f>F11</f>
-        <v/>
-      </c>
-      <c r="J11" s="19">
-        <f>F11-I11</f>
-        <v/>
+      <c r="I11" s="19" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="J11" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K11" s="15" t="n"/>
       <c r="L11" s="15" t="n"/>
@@ -1174,13 +1159,11 @@
           <t>Anen</t>
         </is>
       </c>
-      <c r="I12" s="19">
-        <f>F12</f>
-        <v/>
-      </c>
-      <c r="J12" s="19">
-        <f>F12-I12</f>
-        <v/>
+      <c r="I12" s="19" t="n">
+        <v>600000</v>
+      </c>
+      <c r="J12" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K12" s="15" t="n"/>
       <c r="L12" s="15" t="n"/>
@@ -1234,13 +1217,11 @@
           <t>Susi</t>
         </is>
       </c>
-      <c r="I13" s="19">
-        <f>F13</f>
-        <v/>
-      </c>
-      <c r="J13" s="19">
-        <f>F13-I13</f>
-        <v/>
+      <c r="I13" s="19" t="n">
+        <v>13992000</v>
+      </c>
+      <c r="J13" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K13" s="15" t="n"/>
       <c r="L13" s="15" t="n"/>
@@ -1294,13 +1275,11 @@
           <t>Susi</t>
         </is>
       </c>
-      <c r="I14" s="19">
-        <f>F14</f>
-        <v/>
-      </c>
-      <c r="J14" s="19">
-        <f>F14-I14</f>
-        <v/>
+      <c r="I14" s="19" t="n">
+        <v>8165360</v>
+      </c>
+      <c r="J14" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K14" s="15" t="n"/>
       <c r="L14" s="15" t="n"/>
@@ -1354,13 +1333,11 @@
           <t xml:space="preserve">Eko </t>
         </is>
       </c>
-      <c r="I15" s="19">
-        <f>F15</f>
-        <v/>
-      </c>
-      <c r="J15" s="19">
-        <f>F15-I15</f>
-        <v/>
+      <c r="I15" s="19" t="n">
+        <v>1012500</v>
+      </c>
+      <c r="J15" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K15" s="15" t="n"/>
       <c r="L15" s="15" t="n"/>
@@ -1414,13 +1391,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I16" s="19">
-        <f>F16</f>
-        <v/>
-      </c>
-      <c r="J16" s="19">
-        <f>F16-I16</f>
-        <v/>
+      <c r="I16" s="19" t="n">
+        <v>12278630</v>
+      </c>
+      <c r="J16" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K16" s="15" t="n"/>
       <c r="L16" s="15" t="n"/>
@@ -1474,13 +1449,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I17" s="19">
-        <f>F17</f>
-        <v/>
-      </c>
-      <c r="J17" s="19">
-        <f>F17-I17</f>
-        <v/>
+      <c r="I17" s="19" t="n">
+        <v>8877578</v>
+      </c>
+      <c r="J17" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K17" s="15" t="n"/>
       <c r="L17" s="15" t="n"/>
@@ -1534,13 +1507,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I18" s="19">
-        <f>F18</f>
-        <v/>
-      </c>
-      <c r="J18" s="19">
-        <f>F18-I18</f>
-        <v/>
+      <c r="I18" s="19" t="n">
+        <v>1016100</v>
+      </c>
+      <c r="J18" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K18" s="15" t="n"/>
       <c r="L18" s="15" t="n"/>
@@ -1594,13 +1565,11 @@
           <t>Mail</t>
         </is>
       </c>
-      <c r="I19" s="19">
-        <f>F19</f>
-        <v/>
-      </c>
-      <c r="J19" s="19">
-        <f>F19-I19</f>
-        <v/>
+      <c r="I19" s="19" t="n">
+        <v>7380000</v>
+      </c>
+      <c r="J19" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K19" s="15" t="n"/>
       <c r="L19" s="15" t="n"/>
@@ -1654,13 +1623,11 @@
           <t>Cahaya Alam</t>
         </is>
       </c>
-      <c r="I20" s="19">
-        <f>F20</f>
-        <v/>
-      </c>
-      <c r="J20" s="19">
-        <f>F20-I20</f>
-        <v/>
+      <c r="I20" s="19" t="n">
+        <v>1058000</v>
+      </c>
+      <c r="J20" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K20" s="15" t="n"/>
       <c r="L20" s="15" t="n"/>
@@ -1714,13 +1681,11 @@
           <t>Heni N</t>
         </is>
       </c>
-      <c r="I21" s="19">
-        <f>F21</f>
-        <v/>
-      </c>
-      <c r="J21" s="19">
-        <f>F21-I21</f>
-        <v/>
+      <c r="I21" s="19" t="n">
+        <v>1720000</v>
+      </c>
+      <c r="J21" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K21" s="15" t="n"/>
       <c r="L21" s="15" t="n"/>
@@ -1774,13 +1739,11 @@
           <t>Katering</t>
         </is>
       </c>
-      <c r="I22" s="19">
-        <f>F22</f>
-        <v/>
-      </c>
-      <c r="J22" s="19">
-        <f>F22-I22</f>
-        <v/>
+      <c r="I22" s="19" t="n">
+        <v>2610000</v>
+      </c>
+      <c r="J22" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K22" s="15" t="n"/>
       <c r="L22" s="15" t="n"/>
@@ -1834,13 +1797,11 @@
           <t xml:space="preserve">Eko </t>
         </is>
       </c>
-      <c r="I23" s="19">
-        <f>F23</f>
-        <v/>
-      </c>
-      <c r="J23" s="19">
-        <f>F23-I23</f>
-        <v/>
+      <c r="I23" s="19" t="n">
+        <v>1012500</v>
+      </c>
+      <c r="J23" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K23" s="15" t="n"/>
       <c r="L23" s="15" t="n"/>
@@ -1894,13 +1855,11 @@
           <t>Nurhadi</t>
         </is>
       </c>
-      <c r="I24" s="19">
-        <f>F24</f>
-        <v/>
-      </c>
-      <c r="J24" s="19">
-        <f>F24-I24</f>
-        <v/>
+      <c r="I24" s="19" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="J24" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K24" s="15" t="n"/>
       <c r="L24" s="15" t="n"/>
@@ -1954,13 +1913,11 @@
           <t>Anen</t>
         </is>
       </c>
-      <c r="I25" s="19">
-        <f>F25</f>
-        <v/>
-      </c>
-      <c r="J25" s="19">
-        <f>F25-I25</f>
-        <v/>
+      <c r="I25" s="19" t="n">
+        <v>300000</v>
+      </c>
+      <c r="J25" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K25" s="15" t="n"/>
       <c r="L25" s="15" t="n"/>
@@ -2014,13 +1971,11 @@
           <t>Susi</t>
         </is>
       </c>
-      <c r="I26" s="19">
-        <f>F26</f>
-        <v/>
-      </c>
-      <c r="J26" s="19">
-        <f>F26-I26</f>
-        <v/>
+      <c r="I26" s="19" t="n">
+        <v>3328000</v>
+      </c>
+      <c r="J26" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K26" s="15" t="n"/>
       <c r="L26" s="15" t="n"/>
@@ -2074,13 +2029,11 @@
           <t>Susi</t>
         </is>
       </c>
-      <c r="I27" s="19">
-        <f>F27</f>
-        <v/>
-      </c>
-      <c r="J27" s="19">
-        <f>F27-I27</f>
-        <v/>
+      <c r="I27" s="19" t="n">
+        <v>3399000</v>
+      </c>
+      <c r="J27" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K27" s="15" t="n"/>
       <c r="L27" s="15" t="n"/>
@@ -2134,13 +2087,11 @@
           <t>Susi</t>
         </is>
       </c>
-      <c r="I28" s="19">
-        <f>F28</f>
-        <v/>
-      </c>
-      <c r="J28" s="19">
-        <f>F28-I28</f>
-        <v/>
+      <c r="I28" s="19" t="n">
+        <v>5398000</v>
+      </c>
+      <c r="J28" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K28" s="15" t="n"/>
       <c r="L28" s="15" t="n"/>
@@ -2190,13 +2141,11 @@
         </is>
       </c>
       <c r="H29" s="11" t="n"/>
-      <c r="I29" s="19">
-        <f>F29</f>
-        <v/>
-      </c>
-      <c r="J29" s="19">
-        <f>F29-I29</f>
-        <v/>
+      <c r="I29" s="19" t="n">
+        <v>5248000</v>
+      </c>
+      <c r="J29" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K29" s="15" t="n"/>
       <c r="L29" s="15" t="n"/>
@@ -2246,13 +2195,11 @@
         </is>
       </c>
       <c r="H30" s="11" t="n"/>
-      <c r="I30" s="19">
-        <f>F30</f>
-        <v/>
-      </c>
-      <c r="J30" s="19">
-        <f>F30-I30</f>
-        <v/>
+      <c r="I30" s="19" t="n">
+        <v>5248000</v>
+      </c>
+      <c r="J30" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K30" s="15" t="n"/>
       <c r="L30" s="15" t="n"/>
@@ -2302,13 +2249,11 @@
         </is>
       </c>
       <c r="H31" s="11" t="n"/>
-      <c r="I31" s="19">
-        <f>F31</f>
-        <v/>
-      </c>
-      <c r="J31" s="19">
-        <f>F31-I31</f>
-        <v/>
+      <c r="I31" s="19" t="n">
+        <v>7350000</v>
+      </c>
+      <c r="J31" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K31" s="15" t="n"/>
       <c r="L31" s="15" t="n"/>
@@ -2362,13 +2307,11 @@
           <t>Cahaya Alam</t>
         </is>
       </c>
-      <c r="I32" s="19">
-        <f>F32</f>
-        <v/>
-      </c>
-      <c r="J32" s="19">
-        <f>F32-I32</f>
-        <v/>
+      <c r="I32" s="19" t="n">
+        <v>348000</v>
+      </c>
+      <c r="J32" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K32" s="15" t="n"/>
       <c r="L32" s="15" t="n"/>
@@ -2422,13 +2365,11 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I33" s="19">
-        <f>F33</f>
-        <v/>
-      </c>
-      <c r="J33" s="19">
-        <f>F33-I33</f>
-        <v/>
+      <c r="I33" s="19" t="n">
+        <v>442500</v>
+      </c>
+      <c r="J33" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K33" s="15" t="n"/>
       <c r="L33" s="15" t="n"/>
@@ -2482,13 +2423,11 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I34" s="19">
-        <f>F34</f>
-        <v/>
-      </c>
-      <c r="J34" s="19">
-        <f>F34-I34</f>
-        <v/>
+      <c r="I34" s="19" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="J34" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K34" s="15" t="n"/>
       <c r="L34" s="15" t="n"/>
@@ -2542,13 +2481,11 @@
           <t>Ekky</t>
         </is>
       </c>
-      <c r="I35" s="19">
-        <f>F35</f>
-        <v/>
-      </c>
-      <c r="J35" s="19">
-        <f>F35-I35</f>
-        <v/>
+      <c r="I35" s="19" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J35" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K35" s="15" t="n"/>
       <c r="L35" s="15" t="n"/>
@@ -2602,13 +2539,11 @@
           <t>Ekky</t>
         </is>
       </c>
-      <c r="I36" s="19">
-        <f>F36</f>
-        <v/>
-      </c>
-      <c r="J36" s="19">
-        <f>F36-I36</f>
-        <v/>
+      <c r="I36" s="19" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J36" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K36" s="15" t="n"/>
       <c r="L36" s="15" t="n"/>
@@ -2662,13 +2597,11 @@
           <t>Ekky</t>
         </is>
       </c>
-      <c r="I37" s="19">
-        <f>F37</f>
-        <v/>
-      </c>
-      <c r="J37" s="19">
-        <f>F37-I37</f>
-        <v/>
+      <c r="I37" s="19" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J37" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K37" s="15" t="n"/>
       <c r="L37" s="15" t="n"/>
@@ -2722,13 +2655,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I38" s="19">
-        <f>F38</f>
-        <v/>
-      </c>
-      <c r="J38" s="19">
-        <f>F38-I38</f>
-        <v/>
+      <c r="I38" s="19" t="n">
+        <v>1289000</v>
+      </c>
+      <c r="J38" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K38" s="15" t="n"/>
       <c r="L38" s="15" t="n"/>
@@ -2782,13 +2713,11 @@
           <t>Nurfa</t>
         </is>
       </c>
-      <c r="I39" s="19">
-        <f>F39</f>
-        <v/>
-      </c>
-      <c r="J39" s="19">
-        <f>F39-I39</f>
-        <v/>
+      <c r="I39" s="19" t="n">
+        <v>475865</v>
+      </c>
+      <c r="J39" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K39" s="15" t="n"/>
       <c r="L39" s="15" t="n"/>
@@ -2842,13 +2771,11 @@
           <t>Misbahudin</t>
         </is>
       </c>
-      <c r="I40" s="27">
-        <f>F40</f>
-        <v/>
-      </c>
-      <c r="J40" s="27">
-        <f>F40-I40</f>
-        <v/>
+      <c r="I40" s="27" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="J40" s="27" t="n">
+        <v>0</v>
       </c>
       <c r="K40" s="15" t="n"/>
       <c r="L40" s="15" t="n"/>
@@ -2902,13 +2829,11 @@
           <t>Maxindo</t>
         </is>
       </c>
-      <c r="I41" s="19">
-        <f>F41</f>
-        <v/>
-      </c>
-      <c r="J41" s="19">
-        <f>F41-I41</f>
-        <v/>
+      <c r="I41" s="19" t="n">
+        <v>12765000</v>
+      </c>
+      <c r="J41" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K41" s="15" t="n"/>
       <c r="L41" s="15" t="n"/>
@@ -2958,13 +2883,11 @@
           <t>Abdul Hamid</t>
         </is>
       </c>
-      <c r="I42" s="19">
-        <f>F42</f>
-        <v/>
-      </c>
-      <c r="J42" s="19">
-        <f>F42-I42</f>
-        <v/>
+      <c r="I42" s="19" t="n">
+        <v>8160000</v>
+      </c>
+      <c r="J42" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K42" s="15" t="n"/>
       <c r="L42" s="15" t="n"/>
@@ -3018,13 +2941,11 @@
           <t>PT. Trimitra</t>
         </is>
       </c>
-      <c r="I43" s="19">
-        <f>F43</f>
-        <v/>
-      </c>
-      <c r="J43" s="19">
-        <f>F43-I43</f>
-        <v/>
+      <c r="I43" s="19" t="n">
+        <v>40025000</v>
+      </c>
+      <c r="J43" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K43" s="15" t="n"/>
       <c r="L43" s="15" t="n"/>
@@ -3078,13 +2999,11 @@
           <t>Ekky</t>
         </is>
       </c>
-      <c r="I44" s="19">
-        <f>F44</f>
-        <v/>
-      </c>
-      <c r="J44" s="19">
-        <f>F44-I44</f>
-        <v/>
+      <c r="I44" s="19" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J44" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K44" s="15" t="n"/>
       <c r="L44" s="15" t="n"/>
@@ -3138,13 +3057,11 @@
           <t>Nurfadila</t>
         </is>
       </c>
-      <c r="I45" s="19">
-        <f>F45</f>
-        <v/>
-      </c>
-      <c r="J45" s="19">
-        <f>F45-I45</f>
-        <v/>
+      <c r="I45" s="19" t="n">
+        <v>250460</v>
+      </c>
+      <c r="J45" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K45" s="15" t="n"/>
       <c r="L45" s="15" t="n"/>
@@ -3201,9 +3118,8 @@
       <c r="I46" s="16" t="n">
         <v>1725000</v>
       </c>
-      <c r="J46" s="19">
-        <f>F46-I46</f>
-        <v/>
+      <c r="J46" s="19" t="n">
+        <v>-225000</v>
       </c>
       <c r="K46" s="15" t="n"/>
       <c r="L46" s="15" t="n"/>
@@ -3257,13 +3173,11 @@
           <t>Mael</t>
         </is>
       </c>
-      <c r="I47" s="19">
-        <f>F47</f>
-        <v/>
-      </c>
-      <c r="J47" s="19">
-        <f>F47-I47</f>
-        <v/>
+      <c r="I47" s="19" t="n">
+        <v>1450000</v>
+      </c>
+      <c r="J47" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K47" s="15" t="n"/>
       <c r="L47" s="15" t="n"/>
@@ -3317,13 +3231,11 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I48" s="19">
-        <f>F48</f>
-        <v/>
-      </c>
-      <c r="J48" s="19">
-        <f>F48-I48</f>
-        <v/>
+      <c r="I48" s="19" t="n">
+        <v>300000</v>
+      </c>
+      <c r="J48" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K48" s="15" t="n"/>
       <c r="L48" s="15" t="n"/>
@@ -3377,13 +3289,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I49" s="19">
-        <f>F49</f>
-        <v/>
-      </c>
-      <c r="J49" s="19">
-        <f>F49-I49</f>
-        <v/>
+      <c r="I49" s="19" t="n">
+        <v>213144</v>
+      </c>
+      <c r="J49" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K49" s="15" t="n"/>
       <c r="L49" s="15" t="n"/>
@@ -3437,13 +3347,11 @@
           <t>Cahaya Alam</t>
         </is>
       </c>
-      <c r="I50" s="19">
-        <f>F50</f>
-        <v/>
-      </c>
-      <c r="J50" s="19">
-        <f>F50-I50</f>
-        <v/>
+      <c r="I50" s="19" t="n">
+        <v>541000</v>
+      </c>
+      <c r="J50" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K50" s="15" t="n"/>
       <c r="L50" s="15" t="n"/>
@@ -3497,13 +3405,11 @@
           <t>Cahaya Alam</t>
         </is>
       </c>
-      <c r="I51" s="19">
-        <f>F51</f>
-        <v/>
-      </c>
-      <c r="J51" s="19">
-        <f>F51-I51</f>
-        <v/>
+      <c r="I51" s="19" t="n">
+        <v>775000</v>
+      </c>
+      <c r="J51" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K51" s="15" t="n"/>
       <c r="L51" s="15" t="n"/>
@@ -3557,13 +3463,11 @@
           <t>Said</t>
         </is>
       </c>
-      <c r="I52" s="19">
-        <f>F52</f>
-        <v/>
-      </c>
-      <c r="J52" s="19">
-        <f>F52-I52</f>
-        <v/>
+      <c r="I52" s="19" t="n">
+        <v>225000</v>
+      </c>
+      <c r="J52" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K52" s="15" t="n"/>
       <c r="L52" s="15" t="n"/>
@@ -3617,13 +3521,11 @@
           <t>Said</t>
         </is>
       </c>
-      <c r="I53" s="19">
-        <f>F53</f>
-        <v/>
-      </c>
-      <c r="J53" s="19">
-        <f>F53-I53</f>
-        <v/>
+      <c r="I53" s="19" t="n">
+        <v>259150</v>
+      </c>
+      <c r="J53" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K53" s="15" t="n"/>
       <c r="L53" s="15" t="n"/>
@@ -3677,13 +3579,11 @@
           <t>Aryati Jaya S</t>
         </is>
       </c>
-      <c r="I54" s="19">
-        <f>F54</f>
-        <v/>
-      </c>
-      <c r="J54" s="19">
-        <f>F54-I54</f>
-        <v/>
+      <c r="I54" s="19" t="n">
+        <v>1975000</v>
+      </c>
+      <c r="J54" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K54" s="15" t="n"/>
       <c r="L54" s="15" t="n"/>
@@ -3737,13 +3637,11 @@
           <t>Ekky</t>
         </is>
       </c>
-      <c r="I55" s="19">
-        <f>F55</f>
-        <v/>
-      </c>
-      <c r="J55" s="19">
-        <f>F55-I55</f>
-        <v/>
+      <c r="I55" s="19" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J55" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K55" s="15" t="n"/>
       <c r="L55" s="15" t="n"/>
@@ -3856,9 +3754,8 @@
       <c r="I58" s="16" t="n">
         <v>4272000</v>
       </c>
-      <c r="J58" s="19">
-        <f>F58-I58</f>
-        <v/>
+      <c r="J58" s="19" t="n">
+        <v>228000</v>
       </c>
       <c r="K58" s="15" t="n"/>
       <c r="L58" s="15" t="n"/>
@@ -3915,9 +3812,8 @@
       <c r="I59" s="16" t="n">
         <v>2540515</v>
       </c>
-      <c r="J59" s="19">
-        <f>F59-I59</f>
-        <v/>
+      <c r="J59" s="19" t="n">
+        <v>-540515</v>
       </c>
       <c r="K59" s="15" t="n"/>
       <c r="L59" s="15" t="n"/>
@@ -3971,13 +3867,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I60" s="19">
-        <f>F60</f>
-        <v/>
-      </c>
-      <c r="J60" s="19">
-        <f>F60-I60</f>
-        <v/>
+      <c r="I60" s="19" t="n">
+        <v>3322500</v>
+      </c>
+      <c r="J60" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K60" s="15" t="n"/>
       <c r="L60" s="15" t="n"/>
@@ -4031,13 +3925,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I61" s="19">
-        <f>F61</f>
-        <v/>
-      </c>
-      <c r="J61" s="19">
-        <f>F61-I61</f>
-        <v/>
+      <c r="I61" s="19" t="n">
+        <v>367500</v>
+      </c>
+      <c r="J61" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K61" s="15" t="n"/>
       <c r="L61" s="15" t="n"/>
@@ -4094,9 +3986,8 @@
       <c r="I62" s="16" t="n">
         <v>1178000</v>
       </c>
-      <c r="J62" s="19">
-        <f>F62-I62</f>
-        <v/>
+      <c r="J62" s="19" t="n">
+        <v>822000</v>
       </c>
       <c r="K62" s="15" t="n"/>
       <c r="L62" s="15" t="n"/>
@@ -4153,9 +4044,8 @@
       <c r="I63" s="16" t="n">
         <v>420000</v>
       </c>
-      <c r="J63" s="19">
-        <f>F63-I63</f>
-        <v/>
+      <c r="J63" s="19" t="n">
+        <v>80000</v>
       </c>
       <c r="K63" s="15" t="n"/>
       <c r="L63" s="15" t="n"/>
@@ -4209,13 +4099,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I64" s="19">
-        <f>F64</f>
-        <v/>
-      </c>
-      <c r="J64" s="19">
-        <f>F64-I64</f>
-        <v/>
+      <c r="I64" s="19" t="n">
+        <v>13601829</v>
+      </c>
+      <c r="J64" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K64" s="15" t="n"/>
       <c r="L64" s="15" t="n"/>
@@ -4269,13 +4157,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I65" s="19">
-        <f>F65</f>
-        <v/>
-      </c>
-      <c r="J65" s="19">
-        <f>F65-I65</f>
-        <v/>
+      <c r="I65" s="19" t="n">
+        <v>11881614</v>
+      </c>
+      <c r="J65" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K65" s="15" t="n"/>
       <c r="L65" s="15" t="n"/>
@@ -4329,13 +4215,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I66" s="19">
-        <f>F66</f>
-        <v/>
-      </c>
-      <c r="J66" s="19">
-        <f>F66-I66</f>
-        <v/>
+      <c r="I66" s="19" t="n">
+        <v>1016100</v>
+      </c>
+      <c r="J66" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K66" s="15" t="n"/>
       <c r="L66" s="15" t="n"/>
@@ -4389,13 +4273,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I67" s="19">
-        <f>F67</f>
-        <v/>
-      </c>
-      <c r="J67" s="19">
-        <f>F67-I67</f>
-        <v/>
+      <c r="I67" s="19" t="n">
+        <v>4397500</v>
+      </c>
+      <c r="J67" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K67" s="15" t="n"/>
       <c r="L67" s="15" t="n"/>
@@ -4449,13 +4331,11 @@
           <t>Abdul Hamid</t>
         </is>
       </c>
-      <c r="I68" s="19">
-        <f>F68</f>
-        <v/>
-      </c>
-      <c r="J68" s="19">
-        <f>F68-I68</f>
-        <v/>
+      <c r="I68" s="19" t="n">
+        <v>5455000</v>
+      </c>
+      <c r="J68" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K68" s="15" t="n"/>
       <c r="L68" s="15" t="n"/>
@@ -4509,13 +4389,11 @@
           <t>Anen</t>
         </is>
       </c>
-      <c r="I69" s="19">
-        <f>F69</f>
-        <v/>
-      </c>
-      <c r="J69" s="19">
-        <f>F69-I69</f>
-        <v/>
+      <c r="I69" s="19" t="n">
+        <v>300000</v>
+      </c>
+      <c r="J69" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K69" s="15" t="n"/>
       <c r="L69" s="15" t="n"/>
@@ -4569,13 +4447,11 @@
           <t>Djava Comindo</t>
         </is>
       </c>
-      <c r="I70" s="19">
-        <f>F70</f>
-        <v/>
-      </c>
-      <c r="J70" s="19">
-        <f>F70-I70</f>
-        <v/>
+      <c r="I70" s="19" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="J70" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K70" s="15" t="n"/>
       <c r="L70" s="15" t="n"/>
@@ -4629,13 +4505,11 @@
           <t>Ekky</t>
         </is>
       </c>
-      <c r="I71" s="19">
-        <f>F71</f>
-        <v/>
-      </c>
-      <c r="J71" s="19">
-        <f>F71-I71</f>
-        <v/>
+      <c r="I71" s="19" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J71" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K71" s="15" t="n"/>
       <c r="L71" s="15" t="n"/>
@@ -4689,13 +4563,11 @@
           <t>Koperasi</t>
         </is>
       </c>
-      <c r="I72" s="19">
-        <f>F72</f>
-        <v/>
-      </c>
-      <c r="J72" s="19">
-        <f>F72-I72</f>
-        <v/>
+      <c r="I72" s="19" t="n">
+        <v>4138000</v>
+      </c>
+      <c r="J72" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K72" s="15" t="n"/>
       <c r="L72" s="15" t="n"/>
@@ -4749,13 +4621,11 @@
           <t>Maxindo</t>
         </is>
       </c>
-      <c r="I73" s="19">
-        <f>F73</f>
-        <v/>
-      </c>
-      <c r="J73" s="19">
-        <f>F73-I73</f>
-        <v/>
+      <c r="I73" s="19" t="n">
+        <v>12765000</v>
+      </c>
+      <c r="J73" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K73" s="15" t="n"/>
       <c r="L73" s="15" t="n"/>
@@ -4809,13 +4679,11 @@
           <t>Anen</t>
         </is>
       </c>
-      <c r="I74" s="19">
-        <f>F74</f>
-        <v/>
-      </c>
-      <c r="J74" s="19">
-        <f>F74-I74</f>
-        <v/>
+      <c r="I74" s="19" t="n">
+        <v>5800000</v>
+      </c>
+      <c r="J74" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K74" s="15" t="n"/>
       <c r="L74" s="15" t="n"/>
@@ -4869,13 +4737,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I75" s="19">
-        <f>F75</f>
-        <v/>
-      </c>
-      <c r="J75" s="19">
-        <f>F75-I75</f>
-        <v/>
+      <c r="I75" s="19" t="n">
+        <v>2437500</v>
+      </c>
+      <c r="J75" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K75" s="15" t="n"/>
       <c r="L75" s="15" t="n"/>
@@ -4929,13 +4795,11 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I76" s="19">
-        <f>F76</f>
-        <v/>
-      </c>
-      <c r="J76" s="19">
-        <f>F76-I76</f>
-        <v/>
+      <c r="I76" s="19" t="n">
+        <v>3522500</v>
+      </c>
+      <c r="J76" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K76" s="15" t="n"/>
       <c r="L76" s="15" t="n"/>
@@ -4989,13 +4853,11 @@
           <t>Slamet</t>
         </is>
       </c>
-      <c r="I77" s="19">
-        <f>F77</f>
-        <v/>
-      </c>
-      <c r="J77" s="19">
-        <f>F77-I77</f>
-        <v/>
+      <c r="I77" s="19" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="J77" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K77" s="15" t="n"/>
       <c r="L77" s="15" t="n"/>
@@ -5049,13 +4911,11 @@
           <t>Ekky</t>
         </is>
       </c>
-      <c r="I78" s="19">
-        <f>F78</f>
-        <v/>
-      </c>
-      <c r="J78" s="19">
-        <f>F78-I78</f>
-        <v/>
+      <c r="I78" s="19" t="n">
+        <v>250000</v>
+      </c>
+      <c r="J78" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K78" s="15" t="n"/>
       <c r="L78" s="15" t="n"/>
@@ -5109,13 +4969,11 @@
           <t>Siti Hendrawati</t>
         </is>
       </c>
-      <c r="I79" s="19">
-        <f>F79</f>
-        <v/>
-      </c>
-      <c r="J79" s="19">
-        <f>F79-I79</f>
-        <v/>
+      <c r="I79" s="19" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J79" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K79" s="15" t="n"/>
       <c r="L79" s="15" t="n"/>
@@ -5169,13 +5027,11 @@
           <t>Ekky</t>
         </is>
       </c>
-      <c r="I80" s="19">
-        <f>F80</f>
-        <v/>
-      </c>
-      <c r="J80" s="19">
-        <f>F80-I80</f>
-        <v/>
+      <c r="I80" s="19" t="n">
+        <v>2160000</v>
+      </c>
+      <c r="J80" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K80" s="15" t="n"/>
       <c r="L80" s="15" t="n"/>
@@ -5229,13 +5085,11 @@
           <t>Siti Hendrawati</t>
         </is>
       </c>
-      <c r="I81" s="19">
-        <f>F81</f>
-        <v/>
-      </c>
-      <c r="J81" s="19">
-        <f>F81-I81</f>
-        <v/>
+      <c r="I81" s="19" t="n">
+        <v>4726000</v>
+      </c>
+      <c r="J81" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K81" s="15" t="n"/>
       <c r="L81" s="15" t="n"/>
@@ -5289,13 +5143,11 @@
           <t>Ibu Susi</t>
         </is>
       </c>
-      <c r="I82" s="19">
-        <f>F82</f>
-        <v/>
-      </c>
-      <c r="J82" s="19">
-        <f>F82-I82</f>
-        <v/>
+      <c r="I82" s="19" t="n">
+        <v>1995000</v>
+      </c>
+      <c r="J82" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K82" s="15" t="n"/>
       <c r="L82" s="15" t="n"/>
@@ -5349,13 +5201,11 @@
           <t>Cahaya Alam</t>
         </is>
       </c>
-      <c r="I83" s="19">
-        <f>F83</f>
-        <v/>
-      </c>
-      <c r="J83" s="19">
-        <f>F83-I83</f>
-        <v/>
+      <c r="I83" s="19" t="n">
+        <v>2567000</v>
+      </c>
+      <c r="J83" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K83" s="15" t="n"/>
       <c r="L83" s="15" t="n"/>
@@ -5409,13 +5259,11 @@
           <t>Devyzar Syam</t>
         </is>
       </c>
-      <c r="I84" s="19">
-        <f>F84</f>
-        <v/>
-      </c>
-      <c r="J84" s="19">
-        <f>F84-I84</f>
-        <v/>
+      <c r="I84" s="19" t="n">
+        <v>21000000</v>
+      </c>
+      <c r="J84" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K84" s="15" t="n"/>
       <c r="L84" s="15" t="n"/>
@@ -5469,13 +5317,11 @@
           <t>Cahaya Alam</t>
         </is>
       </c>
-      <c r="I85" s="19">
-        <f>F85</f>
-        <v/>
-      </c>
-      <c r="J85" s="19">
-        <f>F85-I85</f>
-        <v/>
+      <c r="I85" s="19" t="n">
+        <v>1799000</v>
+      </c>
+      <c r="J85" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K85" s="15" t="n"/>
       <c r="L85" s="15" t="n"/>
@@ -5529,13 +5375,11 @@
           <t>Ekky</t>
         </is>
       </c>
-      <c r="I86" s="19">
-        <f>F86</f>
-        <v/>
-      </c>
-      <c r="J86" s="19">
-        <f>F86-I86</f>
-        <v/>
+      <c r="I86" s="19" t="n">
+        <v>350000</v>
+      </c>
+      <c r="J86" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K86" s="15" t="n"/>
       <c r="L86" s="15" t="n"/>
@@ -5589,13 +5433,11 @@
           <t>Asep</t>
         </is>
       </c>
-      <c r="I87" s="27">
-        <f>F87</f>
-        <v/>
-      </c>
-      <c r="J87" s="19">
-        <f>F87-I87</f>
-        <v/>
+      <c r="I87" s="27" t="n">
+        <v>175000500</v>
+      </c>
+      <c r="J87" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K87" s="13" t="n"/>
       <c r="L87" s="13" t="n"/>
@@ -5649,13 +5491,11 @@
           <t>ASep</t>
         </is>
       </c>
-      <c r="I88" s="27">
-        <f>F88</f>
-        <v/>
-      </c>
-      <c r="J88" s="19">
-        <f>F88-I88</f>
-        <v/>
+      <c r="I88" s="27" t="n">
+        <v>15800000</v>
+      </c>
+      <c r="J88" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K88" s="13" t="n"/>
       <c r="L88" s="13" t="n"/>
@@ -5709,13 +5549,11 @@
           <t>Abdul Hamid</t>
         </is>
       </c>
-      <c r="I89" s="19">
-        <f>F89</f>
-        <v/>
-      </c>
-      <c r="J89" s="19">
-        <f>F89-I89</f>
-        <v/>
+      <c r="I89" s="19" t="n">
+        <v>2146000</v>
+      </c>
+      <c r="J89" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K89" s="13" t="n"/>
       <c r="L89" s="13" t="n"/>
@@ -5769,13 +5607,11 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I90" s="19">
-        <f>F90</f>
-        <v/>
-      </c>
-      <c r="J90" s="19">
-        <f>F90-I90</f>
-        <v/>
+      <c r="I90" s="19" t="n">
+        <v>985000</v>
+      </c>
+      <c r="J90" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K90" s="13" t="n"/>
       <c r="L90" s="13" t="n"/>
@@ -5829,13 +5665,11 @@
           <t>Anen</t>
         </is>
       </c>
-      <c r="I91" s="19">
-        <f>F91</f>
-        <v/>
-      </c>
-      <c r="J91" s="19">
-        <f>F91-I91</f>
-        <v/>
+      <c r="I91" s="19" t="n">
+        <v>300000</v>
+      </c>
+      <c r="J91" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K91" s="15" t="n"/>
       <c r="L91" s="15" t="n"/>
@@ -5889,13 +5723,11 @@
           <t>Ekky</t>
         </is>
       </c>
-      <c r="I92" s="19">
-        <f>F92</f>
-        <v/>
-      </c>
-      <c r="J92" s="19">
-        <f>F92-I92</f>
-        <v/>
+      <c r="I92" s="19" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J92" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K92" s="15" t="n"/>
       <c r="L92" s="15" t="n"/>
@@ -5949,13 +5781,11 @@
           <t>Gusti</t>
         </is>
       </c>
-      <c r="I93" s="19">
-        <f>F93</f>
-        <v/>
-      </c>
-      <c r="J93" s="19">
-        <f>F93-I93</f>
-        <v/>
+      <c r="I93" s="19" t="n">
+        <v>3652000</v>
+      </c>
+      <c r="J93" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K93" s="15" t="n"/>
       <c r="L93" s="15" t="n"/>
@@ -6009,13 +5839,11 @@
           <t>Aryati Jaya</t>
         </is>
       </c>
-      <c r="I94" s="19">
-        <f>F94</f>
-        <v/>
-      </c>
-      <c r="J94" s="19">
-        <f>F94-I94</f>
-        <v/>
+      <c r="I94" s="19" t="n">
+        <v>1150000</v>
+      </c>
+      <c r="J94" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K94" s="15" t="n"/>
       <c r="L94" s="15" t="n"/>
@@ -6069,13 +5897,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I95" s="19">
-        <f>F95</f>
-        <v/>
-      </c>
-      <c r="J95" s="19">
-        <f>F95-I95</f>
-        <v/>
+      <c r="I95" s="19" t="n">
+        <v>3354000</v>
+      </c>
+      <c r="J95" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K95" s="15" t="n"/>
       <c r="L95" s="15" t="n"/>
@@ -6129,13 +5955,11 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I96" s="19">
-        <f>F96</f>
-        <v/>
-      </c>
-      <c r="J96" s="19">
-        <f>F96-I96</f>
-        <v/>
+      <c r="I96" s="19" t="n">
+        <v>9156000</v>
+      </c>
+      <c r="J96" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="K96" s="15" t="n"/>
       <c r="L96" s="15" t="n"/>
@@ -6245,9 +6069,8 @@
           <t>Anen</t>
         </is>
       </c>
-      <c r="I99" s="19">
-        <f>F99</f>
-        <v/>
+      <c r="I99" s="19" t="n">
+        <v>300000</v>
       </c>
       <c r="J99" s="15" t="n"/>
       <c r="K99" s="15" t="n"/>
@@ -6302,9 +6125,8 @@
           <t>Masdik</t>
         </is>
       </c>
-      <c r="I100" s="19">
-        <f>F100</f>
-        <v/>
+      <c r="I100" s="19" t="n">
+        <v>29752000</v>
       </c>
       <c r="J100" s="15" t="n"/>
       <c r="K100" s="15" t="n"/>
@@ -6467,9 +6289,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I103" s="19">
-        <f>F103</f>
-        <v/>
+      <c r="I103" s="19" t="n">
+        <v>3322500</v>
       </c>
       <c r="J103" s="15" t="n"/>
       <c r="K103" s="15" t="n"/>
@@ -6524,9 +6345,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I104" s="19">
-        <f>F104</f>
-        <v/>
+      <c r="I104" s="19" t="n">
+        <v>367500</v>
       </c>
       <c r="J104" s="15" t="n"/>
       <c r="K104" s="15" t="n"/>
@@ -6635,9 +6455,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I106" s="19">
-        <f>F106</f>
-        <v/>
+      <c r="I106" s="19" t="n">
+        <v>13907936</v>
       </c>
       <c r="J106" s="15" t="n"/>
       <c r="K106" s="15" t="n"/>
@@ -6692,9 +6511,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I107" s="19">
-        <f>F107</f>
-        <v/>
+      <c r="I107" s="19" t="n">
+        <v>14271606</v>
       </c>
       <c r="J107" s="15" t="n"/>
       <c r="K107" s="15" t="n"/>
@@ -6749,9 +6567,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I108" s="19">
-        <f>F108</f>
-        <v/>
+      <c r="I108" s="19" t="n">
+        <v>1016100</v>
       </c>
       <c r="J108" s="15" t="n"/>
       <c r="K108" s="15" t="n"/>
@@ -6806,9 +6623,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I109" s="19">
-        <f>F109</f>
-        <v/>
+      <c r="I109" s="19" t="n">
+        <v>8903900</v>
       </c>
       <c r="J109" s="15" t="n"/>
       <c r="K109" s="15" t="n"/>
@@ -6863,9 +6679,8 @@
           <t>Katering</t>
         </is>
       </c>
-      <c r="I110" s="19">
-        <f>F110</f>
-        <v/>
+      <c r="I110" s="19" t="n">
+        <v>5117000</v>
       </c>
       <c r="J110" s="15" t="n"/>
       <c r="K110" s="15" t="n"/>
@@ -6920,9 +6735,8 @@
           <t>Abdul Wafi</t>
         </is>
       </c>
-      <c r="I111" s="19">
-        <f>F111</f>
-        <v/>
+      <c r="I111" s="19" t="n">
+        <v>4514250</v>
       </c>
       <c r="J111" s="15" t="n"/>
       <c r="K111" s="15" t="n"/>
@@ -6977,9 +6791,8 @@
           <t>Anen</t>
         </is>
       </c>
-      <c r="I112" s="19">
-        <f>F112</f>
-        <v/>
+      <c r="I112" s="19" t="n">
+        <v>300000</v>
       </c>
       <c r="J112" s="15" t="n"/>
       <c r="K112" s="15" t="n"/>
@@ -7034,9 +6847,8 @@
           <t>Ivan</t>
         </is>
       </c>
-      <c r="I113" s="19">
-        <f>F113</f>
-        <v/>
+      <c r="I113" s="19" t="n">
+        <v>100000000</v>
       </c>
       <c r="J113" s="25" t="n"/>
       <c r="K113" s="25" t="n"/>
@@ -7091,9 +6903,8 @@
           <t>Masdik</t>
         </is>
       </c>
-      <c r="I114" s="19">
-        <f>F114</f>
-        <v/>
+      <c r="I114" s="19" t="n">
+        <v>2000000</v>
       </c>
       <c r="J114" s="15" t="n"/>
       <c r="K114" s="15" t="n"/>
@@ -7148,9 +6959,8 @@
           <t>Endang Hasan</t>
         </is>
       </c>
-      <c r="I115" s="19">
-        <f>F115</f>
-        <v/>
+      <c r="I115" s="19" t="n">
+        <v>9125000</v>
       </c>
       <c r="J115" s="15" t="n"/>
       <c r="K115" s="15" t="n"/>
@@ -7205,9 +7015,8 @@
           <t>Abdul Hamid</t>
         </is>
       </c>
-      <c r="I116" s="19">
-        <f>F116</f>
-        <v/>
+      <c r="I116" s="19" t="n">
+        <v>1340000</v>
       </c>
       <c r="J116" s="15" t="n"/>
       <c r="K116" s="15" t="n"/>
@@ -7262,9 +7071,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I117" s="19">
-        <f>F117</f>
-        <v/>
+      <c r="I117" s="19" t="n">
+        <v>910400</v>
       </c>
       <c r="J117" s="15" t="n"/>
       <c r="K117" s="15" t="n"/>
@@ -7319,9 +7127,8 @@
           <t>Maxindo</t>
         </is>
       </c>
-      <c r="I118" s="19">
-        <f>F118</f>
-        <v/>
+      <c r="I118" s="19" t="n">
+        <v>12765000</v>
       </c>
       <c r="J118" s="15" t="n"/>
       <c r="K118" s="15" t="n"/>
@@ -7376,9 +7183,8 @@
           <t>Ivan</t>
         </is>
       </c>
-      <c r="I119" s="19">
-        <f>F119</f>
-        <v/>
+      <c r="I119" s="19" t="n">
+        <v>9200000</v>
       </c>
       <c r="J119" s="25" t="n"/>
       <c r="K119" s="25" t="inlineStr">
@@ -7441,9 +7247,8 @@
           <t>Hoka</t>
         </is>
       </c>
-      <c r="I120" s="19">
-        <f>F120</f>
-        <v/>
+      <c r="I120" s="19" t="n">
+        <v>1353000</v>
       </c>
       <c r="J120" s="15" t="n"/>
       <c r="K120" s="15" t="n"/>
@@ -7498,9 +7303,8 @@
           <t>Ivan</t>
         </is>
       </c>
-      <c r="I121" s="19">
-        <f>F121</f>
-        <v/>
+      <c r="I121" s="19" t="n">
+        <v>905000</v>
       </c>
       <c r="J121" s="15" t="n"/>
       <c r="K121" s="15" t="n"/>
@@ -7555,9 +7359,8 @@
           <t>Rahmad</t>
         </is>
       </c>
-      <c r="I122" s="19">
-        <f>F122</f>
-        <v/>
+      <c r="I122" s="19" t="n">
+        <v>300000</v>
       </c>
       <c r="J122" s="15" t="n"/>
       <c r="K122" s="15" t="n"/>
@@ -7612,9 +7415,8 @@
           <t>Devyzar Syam</t>
         </is>
       </c>
-      <c r="I123" s="19">
-        <f>F123</f>
-        <v/>
+      <c r="I123" s="19" t="n">
+        <v>21000000</v>
       </c>
       <c r="J123" s="15" t="n"/>
       <c r="K123" s="15" t="n"/>
@@ -7669,9 +7471,8 @@
           <t>Endang Hasan</t>
         </is>
       </c>
-      <c r="I124" s="19">
-        <f>F124</f>
-        <v/>
+      <c r="I124" s="19" t="n">
+        <v>9125000</v>
       </c>
       <c r="J124" s="15" t="n"/>
       <c r="K124" s="15" t="n"/>
@@ -7726,9 +7527,8 @@
           <t>Anen</t>
         </is>
       </c>
-      <c r="I125" s="19">
-        <f>F125</f>
-        <v/>
+      <c r="I125" s="19" t="n">
+        <v>380000</v>
       </c>
       <c r="J125" s="15" t="n"/>
       <c r="K125" s="15" t="n"/>
@@ -7783,9 +7583,8 @@
           <t>Cahaya Alam</t>
         </is>
       </c>
-      <c r="I126" s="19">
-        <f>F126</f>
-        <v/>
+      <c r="I126" s="19" t="n">
+        <v>1970000</v>
       </c>
       <c r="J126" s="15" t="n"/>
       <c r="K126" s="15" t="n"/>
@@ -7840,9 +7639,8 @@
           <t>Susi</t>
         </is>
       </c>
-      <c r="I127" s="19">
-        <f>F127</f>
-        <v/>
+      <c r="I127" s="19" t="n">
+        <v>3591000</v>
       </c>
       <c r="J127" s="15" t="n"/>
       <c r="K127" s="15" t="n"/>
@@ -7897,9 +7695,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I128" s="19">
-        <f>F128</f>
-        <v/>
+      <c r="I128" s="19" t="n">
+        <v>1094000</v>
       </c>
       <c r="J128" s="15" t="n"/>
       <c r="K128" s="15" t="n"/>
@@ -7954,9 +7751,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I129" s="19">
-        <f>F129</f>
-        <v/>
+      <c r="I129" s="19" t="n">
+        <v>388650</v>
       </c>
       <c r="J129" s="15" t="n"/>
       <c r="K129" s="15" t="n"/>
@@ -8011,9 +7807,8 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I130" s="19">
-        <f>F130</f>
-        <v/>
+      <c r="I130" s="19" t="n">
+        <v>4810000</v>
       </c>
       <c r="J130" s="15" t="n"/>
       <c r="K130" s="15" t="n"/>
@@ -8068,9 +7863,8 @@
           <t>Susi</t>
         </is>
       </c>
-      <c r="I131" s="19">
-        <f>F131</f>
-        <v/>
+      <c r="I131" s="19" t="n">
+        <v>13050000</v>
       </c>
       <c r="J131" s="15" t="n"/>
       <c r="K131" s="15" t="n"/>
@@ -8125,9 +7919,8 @@
           <t>Susi</t>
         </is>
       </c>
-      <c r="I132" s="19">
-        <f>F132</f>
-        <v/>
+      <c r="I132" s="19" t="n">
+        <v>838000</v>
       </c>
       <c r="J132" s="15" t="n"/>
       <c r="K132" s="15" t="n"/>
@@ -8182,9 +7975,8 @@
           <t>Susi</t>
         </is>
       </c>
-      <c r="I133" s="19">
-        <f>F133</f>
-        <v/>
+      <c r="I133" s="19" t="n">
+        <v>13035960</v>
       </c>
       <c r="J133" s="15" t="n"/>
       <c r="K133" s="15" t="n"/>
@@ -8239,9 +8031,8 @@
           <t>Bukhori</t>
         </is>
       </c>
-      <c r="I134" s="19">
-        <f>F134</f>
-        <v/>
+      <c r="I134" s="19" t="n">
+        <v>2252500</v>
       </c>
       <c r="J134" s="15" t="n"/>
       <c r="K134" s="15" t="n"/>
@@ -8296,9 +8087,8 @@
           <t>Cahaya Alam</t>
         </is>
       </c>
-      <c r="I135" s="19">
-        <f>F135</f>
-        <v/>
+      <c r="I135" s="19" t="n">
+        <v>1192000</v>
       </c>
       <c r="J135" s="15" t="n"/>
       <c r="K135" s="15" t="n"/>
@@ -8353,9 +8143,8 @@
           <t>Bukhori</t>
         </is>
       </c>
-      <c r="I136" s="19">
-        <f>F136</f>
-        <v/>
+      <c r="I136" s="19" t="n">
+        <v>3002500</v>
       </c>
       <c r="J136" s="15" t="n"/>
       <c r="K136" s="15" t="n"/>
@@ -8410,9 +8199,8 @@
           <t>Syarief</t>
         </is>
       </c>
-      <c r="I137" s="19">
-        <f>F137</f>
-        <v/>
+      <c r="I137" s="19" t="n">
+        <v>350000</v>
       </c>
       <c r="J137" s="15" t="n"/>
       <c r="K137" s="15" t="n"/>
@@ -8467,9 +8255,8 @@
           <t>Ariyati</t>
         </is>
       </c>
-      <c r="I138" s="19">
-        <f>F138</f>
-        <v/>
+      <c r="I138" s="19" t="n">
+        <v>1975000</v>
       </c>
       <c r="J138" s="15" t="n"/>
       <c r="K138" s="15" t="n"/>
@@ -8524,9 +8311,8 @@
           <t>Masdik</t>
         </is>
       </c>
-      <c r="I139" s="19">
-        <f>F139</f>
-        <v/>
+      <c r="I139" s="19" t="n">
+        <v>1550000</v>
       </c>
       <c r="J139" s="15" t="n"/>
       <c r="K139" s="15" t="n"/>
@@ -8581,9 +8367,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I140" s="19">
-        <f>F140</f>
-        <v/>
+      <c r="I140" s="19" t="n">
+        <v>4741610</v>
       </c>
       <c r="J140" s="15" t="n"/>
       <c r="K140" s="15" t="n"/>
@@ -8638,9 +8423,8 @@
           <t>Devzar</t>
         </is>
       </c>
-      <c r="I141" s="19">
-        <f>F141</f>
-        <v/>
+      <c r="I141" s="19" t="n">
+        <v>50000000</v>
       </c>
       <c r="J141" s="15" t="n"/>
       <c r="K141" s="15" t="n"/>
@@ -8695,9 +8479,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I142" s="19">
-        <f>F142</f>
-        <v/>
+      <c r="I142" s="19" t="n">
+        <v>9754000</v>
       </c>
       <c r="J142" s="15" t="n"/>
       <c r="K142" s="15" t="n"/>
@@ -8752,9 +8535,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I143" s="19">
-        <f>F143</f>
-        <v/>
+      <c r="I143" s="19" t="n">
+        <v>8262000</v>
       </c>
       <c r="J143" s="15" t="n"/>
       <c r="K143" s="15" t="n"/>
@@ -8809,9 +8591,8 @@
           <t>Anen</t>
         </is>
       </c>
-      <c r="I144" s="19">
-        <f>F144</f>
-        <v/>
+      <c r="I144" s="19" t="n">
+        <v>420000</v>
       </c>
       <c r="J144" s="15" t="n"/>
       <c r="K144" s="15" t="n"/>
@@ -8866,9 +8647,8 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I145" s="19">
-        <f>F145</f>
-        <v/>
+      <c r="I145" s="19" t="n">
+        <v>1460000</v>
       </c>
       <c r="J145" s="15" t="n"/>
       <c r="K145" s="15" t="n"/>
@@ -8923,9 +8703,8 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I146" s="19">
-        <f>F146</f>
-        <v/>
+      <c r="I146" s="19" t="n">
+        <v>3480000</v>
       </c>
       <c r="J146" s="15" t="n"/>
       <c r="K146" s="15" t="n"/>
@@ -8980,9 +8759,8 @@
           <t>Suryadi</t>
         </is>
       </c>
-      <c r="I147" s="19">
-        <f>F147</f>
-        <v/>
+      <c r="I147" s="19" t="n">
+        <v>6400000</v>
       </c>
       <c r="J147" s="15" t="n"/>
       <c r="K147" s="15" t="n"/>
@@ -9037,9 +8815,8 @@
           <t>Ariyati</t>
         </is>
       </c>
-      <c r="I148" s="19">
-        <f>F148</f>
-        <v/>
+      <c r="I148" s="19" t="n">
+        <v>300000</v>
       </c>
       <c r="J148" s="15" t="n"/>
       <c r="K148" s="15" t="n"/>
@@ -9094,9 +8871,8 @@
           <t>Syarifudin</t>
         </is>
       </c>
-      <c r="I149" s="19">
-        <f>F149</f>
-        <v/>
+      <c r="I149" s="19" t="n">
+        <v>850000</v>
       </c>
       <c r="J149" s="15" t="n"/>
       <c r="K149" s="15" t="n"/>
@@ -9151,9 +8927,8 @@
           <t>Imron</t>
         </is>
       </c>
-      <c r="I150" s="19">
-        <f>F150</f>
-        <v/>
+      <c r="I150" s="19" t="n">
+        <v>1500000</v>
       </c>
       <c r="J150" s="15" t="n"/>
       <c r="K150" s="15" t="n"/>
@@ -9260,9 +9035,8 @@
           <t>Devzar</t>
         </is>
       </c>
-      <c r="I153" s="19">
-        <f>F153</f>
-        <v/>
+      <c r="I153" s="19" t="n">
+        <v>120000000</v>
       </c>
       <c r="J153" s="15" t="n"/>
       <c r="K153" s="15" t="n"/>
@@ -9413,9 +9187,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I156" s="19">
-        <f>F156</f>
-        <v/>
+      <c r="I156" s="19" t="n">
+        <v>3322500</v>
       </c>
       <c r="J156" s="15" t="n"/>
       <c r="K156" s="15" t="n"/>
@@ -9466,9 +9239,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I157" s="19">
-        <f>F157</f>
-        <v/>
+      <c r="I157" s="19" t="n">
+        <v>367500</v>
       </c>
       <c r="J157" s="15" t="n"/>
       <c r="K157" s="15" t="n"/>
@@ -9569,9 +9341,8 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I159" s="19">
-        <f>F159</f>
-        <v/>
+      <c r="I159" s="19" t="n">
+        <v>730000</v>
       </c>
       <c r="J159" s="15" t="n"/>
       <c r="K159" s="15" t="n"/>
@@ -9622,9 +9393,8 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I160" s="19">
-        <f>F160</f>
-        <v/>
+      <c r="I160" s="19" t="n">
+        <v>1560000</v>
       </c>
       <c r="J160" s="15" t="n"/>
       <c r="K160" s="15" t="n"/>
@@ -9675,9 +9445,8 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I161" s="19">
-        <f>F161</f>
-        <v/>
+      <c r="I161" s="19" t="n">
+        <v>1490000</v>
       </c>
       <c r="J161" s="15" t="n"/>
       <c r="K161" s="15" t="n"/>
@@ -9724,9 +9493,8 @@
       </c>
       <c r="G162" s="11" t="n"/>
       <c r="H162" s="11" t="n"/>
-      <c r="I162" s="19">
-        <f>F162</f>
-        <v/>
+      <c r="I162" s="19" t="n">
+        <v>4500000</v>
       </c>
       <c r="J162" s="15" t="n"/>
       <c r="K162" s="15" t="n"/>
@@ -9777,9 +9545,8 @@
           <t>Susi</t>
         </is>
       </c>
-      <c r="I163" s="19">
-        <f>F163</f>
-        <v/>
+      <c r="I163" s="19" t="n">
+        <v>57925000</v>
       </c>
       <c r="J163" s="15" t="n"/>
       <c r="K163" s="15" t="n"/>
@@ -9830,9 +9597,8 @@
           <t>Susi</t>
         </is>
       </c>
-      <c r="I164" s="19">
-        <f>F164</f>
-        <v/>
+      <c r="I164" s="19" t="n">
+        <v>1958294</v>
       </c>
       <c r="J164" s="15" t="n"/>
       <c r="K164" s="15" t="n"/>
@@ -9879,9 +9645,8 @@
       </c>
       <c r="G165" s="11" t="n"/>
       <c r="H165" s="11" t="n"/>
-      <c r="I165" s="19">
-        <f>F165</f>
-        <v/>
+      <c r="I165" s="19" t="n">
+        <v>550000</v>
       </c>
       <c r="J165" s="15" t="n"/>
       <c r="K165" s="15" t="n"/>
@@ -9932,9 +9697,8 @@
           <t>Cahaya Alam</t>
         </is>
       </c>
-      <c r="I166" s="19">
-        <f>F166</f>
-        <v/>
+      <c r="I166" s="19" t="n">
+        <v>3220000</v>
       </c>
       <c r="J166" s="15" t="n"/>
       <c r="K166" s="15" t="n"/>
@@ -9981,9 +9745,8 @@
       </c>
       <c r="G167" s="11" t="n"/>
       <c r="H167" s="11" t="n"/>
-      <c r="I167" s="19">
-        <f>F167</f>
-        <v/>
+      <c r="I167" s="19" t="n">
+        <v>4862000</v>
       </c>
       <c r="J167" s="15" t="n"/>
       <c r="K167" s="15" t="n"/>
@@ -10034,9 +9797,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I168" s="19">
-        <f>F168</f>
-        <v/>
+      <c r="I168" s="19" t="n">
+        <v>16628392</v>
       </c>
       <c r="J168" s="15" t="n"/>
       <c r="K168" s="15" t="n"/>
@@ -10087,9 +9849,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I169" s="19">
-        <f>F169</f>
-        <v/>
+      <c r="I169" s="19" t="n">
+        <v>15661549</v>
       </c>
       <c r="J169" s="15" t="n"/>
       <c r="K169" s="15" t="n"/>
@@ -10140,9 +9901,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I170" s="19">
-        <f>F170</f>
-        <v/>
+      <c r="I170" s="19" t="n">
+        <v>1018875</v>
       </c>
       <c r="J170" s="15" t="n"/>
       <c r="K170" s="15" t="n"/>
@@ -10189,9 +9949,8 @@
       </c>
       <c r="G171" s="11" t="n"/>
       <c r="H171" s="11" t="n"/>
-      <c r="I171" s="19">
-        <f>F171</f>
-        <v/>
+      <c r="I171" s="19" t="n">
+        <v>2942000</v>
       </c>
       <c r="J171" s="15" t="n"/>
       <c r="K171" s="15" t="n"/>
@@ -10238,9 +9997,8 @@
       </c>
       <c r="G172" s="11" t="n"/>
       <c r="H172" s="11" t="n"/>
-      <c r="I172" s="19">
-        <f>F172</f>
-        <v/>
+      <c r="I172" s="19" t="n">
+        <v>1153900</v>
       </c>
       <c r="J172" s="15" t="n"/>
       <c r="K172" s="15" t="n"/>
@@ -10291,9 +10049,8 @@
           <t>Rinni</t>
         </is>
       </c>
-      <c r="I173" s="19">
-        <f>F173</f>
-        <v/>
+      <c r="I173" s="19" t="n">
+        <v>5185000</v>
       </c>
       <c r="J173" s="15" t="n"/>
       <c r="K173" s="15" t="n"/>
@@ -10344,9 +10101,8 @@
           <t>Bengkel Mobil</t>
         </is>
       </c>
-      <c r="I174" s="19">
-        <f>F174</f>
-        <v/>
+      <c r="I174" s="19" t="n">
+        <v>1045000</v>
       </c>
       <c r="J174" s="15" t="n"/>
       <c r="K174" s="15" t="n"/>
@@ -10393,9 +10149,8 @@
       </c>
       <c r="G175" s="11" t="n"/>
       <c r="H175" s="11" t="n"/>
-      <c r="I175" s="19">
-        <f>F175</f>
-        <v/>
+      <c r="I175" s="19" t="n">
+        <v>1055000</v>
       </c>
       <c r="J175" s="15" t="n"/>
       <c r="K175" s="15" t="n"/>
@@ -10446,9 +10201,8 @@
           <t>Maxindo</t>
         </is>
       </c>
-      <c r="I176" s="19">
-        <f>F176</f>
-        <v/>
+      <c r="I176" s="19" t="n">
+        <v>12765000</v>
       </c>
       <c r="J176" s="15" t="n"/>
       <c r="K176" s="15" t="n"/>
@@ -10499,9 +10253,8 @@
           <t>Devyzar Syam</t>
         </is>
       </c>
-      <c r="I177" s="19">
-        <f>F177</f>
-        <v/>
+      <c r="I177" s="19" t="n">
+        <v>10000000</v>
       </c>
       <c r="J177" s="15" t="n"/>
       <c r="K177" s="15" t="n"/>
@@ -10552,9 +10305,8 @@
           <t>Eko</t>
         </is>
       </c>
-      <c r="I178" s="19">
-        <f>F178</f>
-        <v/>
+      <c r="I178" s="19" t="n">
+        <v>1080000</v>
       </c>
       <c r="J178" s="15" t="n"/>
       <c r="K178" s="15" t="n"/>
@@ -10605,9 +10357,8 @@
           <t>Hannochs</t>
         </is>
       </c>
-      <c r="I179" s="19">
-        <f>F179</f>
-        <v/>
+      <c r="I179" s="19" t="n">
+        <v>1589400</v>
       </c>
       <c r="J179" s="15" t="n"/>
       <c r="K179" s="15" t="n"/>
@@ -10658,9 +10409,8 @@
           <t>Cahaya Alam</t>
         </is>
       </c>
-      <c r="I180" s="19">
-        <f>F180</f>
-        <v/>
+      <c r="I180" s="19" t="n">
+        <v>1206000</v>
       </c>
       <c r="J180" s="15" t="n"/>
       <c r="K180" s="15" t="n"/>
@@ -10707,9 +10457,8 @@
       </c>
       <c r="G181" s="11" t="n"/>
       <c r="H181" s="11" t="n"/>
-      <c r="I181" s="19">
-        <f>F181</f>
-        <v/>
+      <c r="I181" s="19" t="n">
+        <v>550000</v>
       </c>
       <c r="J181" s="15" t="n"/>
       <c r="K181" s="15" t="n"/>
@@ -10760,9 +10509,8 @@
           <t>Masdik</t>
         </is>
       </c>
-      <c r="I182" s="19">
-        <f>F182</f>
-        <v/>
+      <c r="I182" s="19" t="n">
+        <v>4546000</v>
       </c>
       <c r="J182" s="15" t="n"/>
       <c r="K182" s="15" t="n"/>
@@ -10813,9 +10561,8 @@
           <t>Ariyati</t>
         </is>
       </c>
-      <c r="I183" s="19">
-        <f>F183</f>
-        <v/>
+      <c r="I183" s="19" t="n">
+        <v>2295000</v>
       </c>
       <c r="J183" s="15" t="n"/>
       <c r="K183" s="15" t="n"/>

</xml_diff>